<commit_message>
v0.8 add_table_set_default_col, add_table_set new
</commit_message>
<xml_diff>
--- a/mode_docx_gen/pmi_dzt/part/tdif/hf2phar1/HF2PHAR1.xlsx
+++ b/mode_docx_gen/pmi_dzt/part/tdif/hf2phar1/HF2PHAR1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="107">
   <si>
     <t>Категория (group)</t>
   </si>
@@ -163,9 +163,6 @@
     <t>FLOAT32</t>
   </si>
   <si>
-    <t>%</t>
-  </si>
-  <si>
     <t>ASG</t>
   </si>
   <si>
@@ -253,9 +250,6 @@
     <t>Выдержка времени ввода перекрестной блокировки</t>
   </si>
   <si>
-    <t>с</t>
-  </si>
-  <si>
     <t>CrossBlkDlTmms</t>
   </si>
   <si>
@@ -329,6 +323,24 @@
   </si>
   <si>
     <t>Ratio</t>
+  </si>
+  <si>
+    <t>мс</t>
+  </si>
+  <si>
+    <t>о.е.</t>
+  </si>
+  <si>
+    <t>0.1</t>
+  </si>
+  <si>
+    <t>0.5</t>
+  </si>
+  <si>
+    <t>0.01</t>
+  </si>
+  <si>
+    <t>0.13</t>
   </si>
 </sst>
 </file>
@@ -351,7 +363,7 @@
       <charset val="204"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -379,6 +391,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -434,7 +452,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -449,6 +467,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -761,6 +780,7 @@
     <col min="5" max="5" width="17.42578125" customWidth="1"/>
     <col min="6" max="6" width="23.42578125" customWidth="1"/>
     <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="17.5703125" customWidth="1"/>
     <col min="27" max="27" width="14.28515625" customWidth="1"/>
     <col min="28" max="28" width="22.5703125" customWidth="1"/>
   </cols>
@@ -857,7 +877,7 @@
         <v>29</v>
       </c>
       <c r="AE1" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -865,46 +885,46 @@
         <v>44</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="N2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="I2" s="3">
-        <v>10</v>
-      </c>
-      <c r="J2" s="3">
-        <v>50</v>
-      </c>
-      <c r="K2" s="3">
-        <v>1</v>
-      </c>
-      <c r="L2" s="3">
-        <v>13</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>49</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>46</v>
@@ -913,7 +933,7 @@
         <v>32</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>39</v>
@@ -940,10 +960,10 @@
         <v>0</v>
       </c>
       <c r="AA2" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AC2" s="3" t="s">
         <v>32</v>
@@ -952,7 +972,7 @@
         <v>32</v>
       </c>
       <c r="AE2" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -960,55 +980,55 @@
         <v>44</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0</v>
+      </c>
+      <c r="J3" s="3">
+        <v>1</v>
+      </c>
+      <c r="K3" s="3">
+        <v>1</v>
+      </c>
+      <c r="L3" s="3">
+        <v>0</v>
+      </c>
+      <c r="M3" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
-      <c r="J3" s="3">
-        <v>1</v>
-      </c>
-      <c r="K3" s="3">
-        <v>1</v>
-      </c>
-      <c r="L3" s="3">
-        <v>0</v>
-      </c>
-      <c r="M3" s="3" t="s">
+      <c r="N3" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="O3" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="O3" s="3" t="s">
-        <v>71</v>
-      </c>
       <c r="P3" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q3" s="3" t="s">
         <v>32</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S3" s="3" t="s">
         <v>39</v>
@@ -1035,10 +1055,10 @@
         <v>0</v>
       </c>
       <c r="AA3" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB3" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="AB3" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="AC3" s="3" t="s">
         <v>32</v>
@@ -1052,55 +1072,55 @@
         <v>44</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="I4" s="8">
+        <v>60</v>
+      </c>
+      <c r="J4" s="8">
+        <v>4000</v>
+      </c>
+      <c r="K4" s="8">
+        <v>10</v>
+      </c>
+      <c r="L4" s="8">
+        <v>60</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G4" s="3" t="s">
+      <c r="N4" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="I4" s="3">
-        <v>0.06</v>
-      </c>
-      <c r="J4" s="3">
-        <v>4</v>
-      </c>
-      <c r="K4" s="3">
-        <v>0.01</v>
-      </c>
-      <c r="L4" s="3">
-        <v>0.06</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="N4" s="3" t="s">
-        <v>75</v>
-      </c>
       <c r="O4" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Q4" s="3" t="s">
         <v>32</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S4" s="3" t="s">
         <v>39</v>
@@ -1127,10 +1147,10 @@
         <v>0</v>
       </c>
       <c r="AA4" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AB4" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="AC4" s="3" t="s">
         <v>32</v>
@@ -1139,7 +1159,7 @@
         <v>32</v>
       </c>
       <c r="AE4" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1147,41 +1167,41 @@
         <v>44</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="I5" s="8">
+        <v>0</v>
+      </c>
+      <c r="J5" s="8">
+        <v>100</v>
+      </c>
+      <c r="K5" s="8">
+        <v>1</v>
+      </c>
+      <c r="L5" s="8">
+        <v>15</v>
+      </c>
+      <c r="M5" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="I5" s="3">
-        <v>0</v>
-      </c>
-      <c r="J5" s="3">
-        <v>0.1</v>
-      </c>
-      <c r="K5" s="3">
-        <v>1E-3</v>
-      </c>
-      <c r="L5" s="3">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>69</v>
-      </c>
       <c r="N5" s="3" t="s">
         <v>32</v>
       </c>
@@ -1222,7 +1242,7 @@
         <v>0</v>
       </c>
       <c r="AA5" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AB5" s="3" t="s">
         <v>32</v>
@@ -1234,7 +1254,7 @@
         <v>32</v>
       </c>
       <c r="AE5" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1242,10 +1262,10 @@
         <v>30</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>31</v>
@@ -1275,7 +1295,7 @@
         <v>32</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="N6" s="3" t="s">
         <v>34</v>
@@ -1317,7 +1337,7 @@
         <v>0</v>
       </c>
       <c r="AA6" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AB6" s="3" t="s">
         <v>40</v>
@@ -1334,10 +1354,10 @@
         <v>30</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>41</v>
@@ -1367,7 +1387,7 @@
         <v>32</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="N7" s="3" t="s">
         <v>34</v>
@@ -1409,7 +1429,7 @@
         <v>0</v>
       </c>
       <c r="AA7" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AB7" s="3" t="s">
         <v>43</v>
@@ -1426,49 +1446,49 @@
         <v>30</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M8" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G8" s="3" t="s">
+      <c r="N8" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="N8" s="3" t="s">
+      <c r="O8" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="O8" s="3" t="s">
+      <c r="P8" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="P8" s="3" t="s">
-        <v>55</v>
       </c>
       <c r="Q8" s="3" t="s">
         <v>32</v>
@@ -1501,10 +1521,10 @@
         <v>1</v>
       </c>
       <c r="AA8" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AB8" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AC8" s="3" t="s">
         <v>32</v>
@@ -1518,49 +1538,49 @@
         <v>30</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M9" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G9" s="3" t="s">
+      <c r="N9" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="N9" s="3" t="s">
-        <v>53</v>
-      </c>
       <c r="O9" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q9" s="3" t="s">
         <v>32</v>
@@ -1593,10 +1613,10 @@
         <v>1</v>
       </c>
       <c r="AA9" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AB9" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AC9" s="3" t="s">
         <v>32</v>
@@ -1610,49 +1630,49 @@
         <v>30</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M10" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="N10" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="O10" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="N10" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>91</v>
-      </c>
       <c r="P10" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q10" s="3" t="s">
         <v>32</v>
@@ -1685,10 +1705,10 @@
         <v>1</v>
       </c>
       <c r="AA10" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AB10" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AC10" s="3" t="s">
         <v>32</v>
@@ -1702,49 +1722,49 @@
         <v>30</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M11" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D11" s="3" t="s">
+      <c r="N11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="O11" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="M11" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="N11" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="O11" s="3" t="s">
-        <v>92</v>
-      </c>
       <c r="P11" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q11" s="3" t="s">
         <v>32</v>
@@ -1777,10 +1797,10 @@
         <v>1</v>
       </c>
       <c r="AA11" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AB11" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AC11" s="3" t="s">
         <v>32</v>
@@ -1808,44 +1828,44 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" t="s">
         <v>96</v>
-      </c>
-      <c r="B5" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B6">
         <v>30</v>

</xml_diff>